<commit_message>
data: update 고객사계측기현황.xlsx for 2026-09-10
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사계측기현황.xlsx
+++ b/docs/dashboard/data/고객사계측기현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -174,30 +174,30 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하이에어코리아(주)</t>
+          <t>굴드펌프(주)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>경상남도 김해시</t>
+          <t>충청북도 청주시 흥덕구</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>6038110081</t>
+          <t>2118642792</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11.0</v>
+        <v>0.0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>11.0</v>
+        <v>0.0</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>438.0</v>
+        <v>190.0</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.0</v>
@@ -217,30 +217,30 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>보그워너충주 유한책임회사</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>충청북도 충주시</t>
+          <t>경상남도 김해시</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>3038108176</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>284.0</v>
+        <v>429.0</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0.0</v>
@@ -260,30 +260,30 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>보그워너충주 유한책임회사</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>경기도 성남시 수정구</t>
+          <t>충청북도 충주시</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>3038108176</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>182.0</v>
+        <v>284.0</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0.0</v>
@@ -303,30 +303,30 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>현대건설(주)</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>경상북도 울진군</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1018116293</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4.0</v>
+        <v>10.0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>4.0</v>
+        <v>10.0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2.0</v>
+        <v>10.0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30.0</v>
+        <v>178.0</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0.0</v>
@@ -346,30 +346,30 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>19.0</v>
+        <v>30.0</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0.0</v>
@@ -389,17 +389,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -412,7 +412,7 @@
         <v>0.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>53.0</v>
+        <v>19.0</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0.0</v>
@@ -432,17 +432,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -455,7 +455,7 @@
         <v>0.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>190.0</v>
+        <v>53.0</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0.0</v>
@@ -475,17 +475,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -498,7 +498,7 @@
         <v>0.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>37.0</v>
+        <v>190.0</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>0.0</v>
@@ -518,7 +518,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -528,29 +528,29 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>293.0</v>
+        <v>0.0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>293.0</v>
+        <v>0.0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>54.0</v>
+        <v>0.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>179.0</v>
+        <v>40.0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>23.0</v>
+        <v>0.0</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>21.0</v>
+        <v>0.0</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>226.0</v>
+        <v>0.0</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -571,29 +571,29 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.0</v>
+        <v>54.0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>223.0</v>
+        <v>179.0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.0</v>
+        <v>21.0</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.0</v>
+        <v>226.0</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -604,17 +604,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
@@ -627,7 +627,7 @@
         <v>0.0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>23.0</v>
+        <v>223.0</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0.0</v>
@@ -647,17 +647,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -670,7 +670,7 @@
         <v>0.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>81.0</v>
+        <v>23.0</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0.0</v>
@@ -690,17 +690,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -713,7 +713,7 @@
         <v>0.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>118.0</v>
+        <v>62.0</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0.0</v>
@@ -733,17 +733,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -756,7 +756,7 @@
         <v>0.0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>49.0</v>
+        <v>118.0</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>0.0</v>
@@ -776,17 +776,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -799,7 +799,7 @@
         <v>0.0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>19.0</v>
+        <v>49.0</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0.0</v>
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -842,7 +842,7 @@
         <v>0.0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>58.0</v>
+        <v>19.0</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>0.0</v>
@@ -862,7 +862,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -885,7 +885,7 @@
         <v>0.0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>9.0</v>
+        <v>58.0</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0.0</v>
@@ -905,17 +905,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
@@ -928,7 +928,7 @@
         <v>0.0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>12.0</v>
+        <v>9.0</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>0.0</v>
@@ -948,17 +948,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -971,7 +971,7 @@
         <v>0.0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>70.0</v>
+        <v>12.0</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>0.0</v>
@@ -991,30 +991,30 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>82.0</v>
+        <v>70.0</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>0.0</v>
@@ -1034,30 +1034,30 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>37.0</v>
+        <v>82.0</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>0.0</v>
@@ -1077,7 +1077,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -1100,7 +1100,7 @@
         <v>0.0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>47.0</v>
+        <v>37.0</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>0.0</v>
@@ -1120,7 +1120,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1130,20 +1130,20 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>80.0</v>
+        <v>0.0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>80.0</v>
+        <v>0.0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>47.0</v>
+        <v>0.0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>44.0</v>
+        <v>79.0</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>0.0</v>
@@ -1163,30 +1163,30 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>288.0</v>
+        <v>80.0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>288.0</v>
+        <v>80.0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1.0</v>
+        <v>47.0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>217.0</v>
+        <v>44.0</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>0.0</v>
@@ -1195,7 +1195,7 @@
         <v>0.0</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>73.0</v>
+        <v>0.0</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1206,30 +1206,30 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>47.0</v>
+        <v>288.0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>47.0</v>
+        <v>288.0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>27.0</v>
+        <v>217.0</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>0.0</v>
@@ -1238,7 +1238,7 @@
         <v>0.0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.0</v>
+        <v>73.0</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1249,39 +1249,39 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>209.0</v>
+        <v>47.0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>209.0</v>
+        <v>47.0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>92.0</v>
+        <v>10.0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>123.0</v>
+        <v>27.0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>11.0</v>
+        <v>0.0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1292,39 +1292,39 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>157.0</v>
+        <v>209.0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>157.0</v>
+        <v>209.0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1.0</v>
+        <v>92.0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>107.0</v>
+        <v>122.0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>2.0</v>
+        <v>11.0</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>7.0</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>64.0</v>
+        <v>13.0</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -1335,39 +1335,39 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>70.0</v>
+        <v>157.0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>70.0</v>
+        <v>157.0</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>70.0</v>
+        <v>94.0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>17.0</v>
+        <v>2.0</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>50.0</v>
+        <v>71.0</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -1378,39 +1378,39 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>103.0</v>
+        <v>70.0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="I30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.0</v>
+        <v>49.0</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -1421,36 +1421,36 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>174.0</v>
+        <v>103.0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.0</v>
+        <v>0.0</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.0</v>
@@ -1464,39 +1464,39 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.0</v>
+        <v>194.0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0</v>
+        <v>194.0</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>35.0</v>
+        <v>169.0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -1507,17 +1507,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
@@ -1530,7 +1530,7 @@
         <v>0.0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>286.0</v>
+        <v>35.0</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>0.0</v>
@@ -1550,30 +1550,30 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>70.0</v>
+        <v>286.0</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>0.0</v>
@@ -1593,39 +1593,39 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>452.0</v>
+        <v>5.0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>315.0</v>
+        <v>5.0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>243.0</v>
+        <v>70.0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>18.0</v>
+        <v>0.0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>48.0</v>
+        <v>1.0</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -1636,39 +1636,39 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.0</v>
+        <v>452.0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.0</v>
+        <v>315.0</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G36" s="2" t="n">
+        <v>234.0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="I36" s="2" t="n">
         <v>41.0</v>
       </c>
-      <c r="H36" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I36" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="J36" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -1679,30 +1679,30 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>163.0</v>
+        <v>0.0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>163.0</v>
+        <v>0.0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>10.0</v>
+        <v>41.0</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>0.0</v>
@@ -1722,30 +1722,30 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>45.0</v>
+        <v>163.0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>45.0</v>
+        <v>163.0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>150.0</v>
+        <v>10.0</v>
       </c>
       <c r="H38" s="2" t="n">
         <v>0.0</v>
@@ -1765,39 +1765,39 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>237.0</v>
+        <v>45.0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>237.0</v>
+        <v>45.0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>57.0</v>
+        <v>0.0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>183.0</v>
+        <v>150.0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>30.0</v>
+        <v>0.0</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>27.0</v>
+        <v>0.0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>86.0</v>
+        <v>0.0</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -1808,39 +1808,39 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>10.0</v>
+        <v>237.0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>10.0</v>
+        <v>237.0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.0</v>
+        <v>57.0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>160.0</v>
+        <v>183.0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.0</v>
+        <v>86.0</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -1851,39 +1851,39 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>23.0</v>
+        <v>160.0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -1894,39 +1894,39 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1827.0</v>
+        <v>60.0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1827.0</v>
+        <v>60.0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>525.0</v>
+        <v>16.0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>936.0</v>
+        <v>23.0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>18.0</v>
+        <v>2.0</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -1937,39 +1937,39 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>84.0</v>
+        <v>1827.0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>84.0</v>
+        <v>1827.0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>22.0</v>
+        <v>525.0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>70.0</v>
+        <v>936.0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -1980,36 +1980,36 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1183.0</v>
+        <v>84.0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1164.0</v>
+        <v>84.0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>28.0</v>
+        <v>22.0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1523.0</v>
+        <v>70.0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>37.0</v>
+        <v>0.0</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.0</v>
@@ -2023,39 +2023,39 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>경남 창원시 성산구</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>614.0</v>
+        <v>1184.0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>614.0</v>
+        <v>1165.0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>250.0</v>
+        <v>28.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>309.0</v>
+        <v>1521.0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>9.0</v>
+        <v>39.0</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>376.0</v>
+        <v>0.0</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -2066,39 +2066,39 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>충북 음성군</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>916.0</v>
+        <v>614.0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>916.0</v>
+        <v>614.0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>128.0</v>
+        <v>250.0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>871.0</v>
+        <v>319.0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>41.0</v>
+        <v>2.0</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>42.0</v>
+        <v>9.0</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>145.0</v>
+        <v>376.0</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -2109,41 +2109,84 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>(주)휴니드테크놀러지스</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>인천 연수구</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>1238106174</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>128.0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>839.0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>117.0</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>21.0</v>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>163.0</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>(주)서연이화 아산공장</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>충남 아산시</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>3128564374</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n">
+      <c r="D48" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="E47" s="2" t="n">
+      <c r="E48" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="F48" s="2" t="n">
         <v>5.0</v>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="H47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
data: update 고객사계측기현황.xlsx for 2026-09-18
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사계측기현황.xlsx
+++ b/docs/dashboard/data/고객사계측기현황.xlsx
@@ -98,20 +98,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
     <col min="2" max="2" width="18.0" customWidth="true"/>
     <col min="3" max="3" width="15.0" customWidth="true"/>
-    <col min="4" max="4" width="10.0" customWidth="true"/>
-    <col min="5" max="5" width="12.0" customWidth="true"/>
-    <col min="6" max="6" width="10.0" customWidth="true"/>
+    <col min="4" max="4" width="16.0" customWidth="true"/>
+    <col min="5" max="5" width="10.0" customWidth="true"/>
+    <col min="6" max="6" width="12.0" customWidth="true"/>
     <col min="7" max="7" width="10.0" customWidth="true"/>
     <col min="8" max="8" width="10.0" customWidth="true"/>
     <col min="9" max="9" width="10.0" customWidth="true"/>
     <col min="10" max="10" width="10.0" customWidth="true"/>
     <col min="11" max="11" width="10.0" customWidth="true"/>
+    <col min="12" max="12" width="10.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -132,40 +133,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>영업 담당자</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>총자산</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>성적서 대상</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>미매핑</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>KIC 연간</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>교정 준비</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>교정 임박</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>기한 초과</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -174,21 +180,23 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>굴드펌프(주)</t>
+          <t>한국의료기기평가원</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>충청북도 청주시 흥덕구</t>
+          <t>경기도 성남시 분당구</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2118642792</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.0</v>
+          <t>1298210386</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>한윤규 외 1명</t>
+        </is>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.0</v>
@@ -197,10 +205,10 @@
         <v>0.0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>190.0</v>
+        <v>0.0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.0</v>
+        <v>136.0</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0.0</v>
@@ -208,7 +216,10 @@
       <c r="J2" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -217,41 +228,46 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>하이에어코리아(주)</t>
+          <t>굴드펌프(주)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>경상남도 김해시</t>
+          <t>충청북도 청주시 흥덕구</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>6038110081</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>11.0</v>
+          <t>2118642792</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>이선재 외 1명</t>
+        </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>11.0</v>
+        <v>16.0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>429.0</v>
+        <v>7.0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.0</v>
+        <v>192.0</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
+        <v>3.0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -260,41 +276,46 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>보그워너충주 유한책임회사</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>충청북도 충주시</t>
+          <t>경상남도 김해시</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>3038108176</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.0</v>
+          <t>6038110081</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>한규범 외 5명</t>
+        </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0</v>
+        <v>467.0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.0</v>
+        <v>467.0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>284.0</v>
+        <v>15.0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.0</v>
+        <v>421.0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.0</v>
+        <v>24.0</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+        <v>15.0</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>136.0</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -316,28 +337,33 @@
           <t>1298603001</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>한윤규</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>119.0</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>99.0</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>99.0</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>178.0</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>10.0</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>178.0</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -359,28 +385,33 @@
           <t>1018116293</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>4.0</v>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E6" s="2" t="n">
         <v>4.0</v>
       </c>
       <c r="F6" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>2.0</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>30.0</v>
       </c>
-      <c r="H6" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I6" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -402,8 +433,10 @@
           <t>6068641818</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>0.0</v>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>송민규 외 5명</t>
+        </is>
       </c>
       <c r="E7" s="2" t="n">
         <v>0.0</v>
@@ -412,18 +445,21 @@
         <v>0.0</v>
       </c>
       <c r="G7" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>19.0</v>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I7" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -445,8 +481,10 @@
           <t>1048644532</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>0.0</v>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E8" s="2" t="n">
         <v>0.0</v>
@@ -455,10 +493,10 @@
         <v>0.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>53.0</v>
+        <v>0.0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.0</v>
+        <v>37.0</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0.0</v>
@@ -466,7 +504,10 @@
       <c r="J8" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -488,20 +529,22 @@
           <t>2218802452</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
-        <v>0.0</v>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>전원준 외 1명</t>
+        </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>190.0</v>
+        <v>6.0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.0</v>
+        <v>166.0</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0.0</v>
@@ -509,7 +552,10 @@
       <c r="J9" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -531,28 +577,33 @@
           <t>1408121883</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>0.0</v>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0</v>
+        <v>44.0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.0</v>
+        <v>44.0</v>
       </c>
       <c r="G10" s="2" t="n">
+        <v>43.0</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>40.0</v>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I10" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -574,28 +625,33 @@
           <t>3128545076</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>293.0</v>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E11" s="2" t="n">
         <v>293.0</v>
       </c>
       <c r="F11" s="2" t="n">
+        <v>293.0</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>54.0</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>179.0</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>27.0</v>
+        <v>231.0</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>21.0</v>
+        <v>30.0</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>226.0</v>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+        <v>19.0</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>227.0</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -617,8 +673,10 @@
           <t>7398801954</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>0.0</v>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E12" s="2" t="n">
         <v>0.0</v>
@@ -627,18 +685,21 @@
         <v>0.0</v>
       </c>
       <c r="G12" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>223.0</v>
       </c>
-      <c r="H12" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I12" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -660,8 +721,10 @@
           <t>8858800321</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
-        <v>0.0</v>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E13" s="2" t="n">
         <v>0.0</v>
@@ -670,18 +733,21 @@
         <v>0.0</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>23.0</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I13" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -703,8 +769,10 @@
           <t>7888101296</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
-        <v>0.0</v>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E14" s="2" t="n">
         <v>0.0</v>
@@ -713,10 +781,10 @@
         <v>0.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>62.0</v>
+        <v>0.0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>0.0</v>
@@ -724,7 +792,10 @@
       <c r="J14" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -746,8 +817,10 @@
           <t>5318701197</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
-        <v>0.0</v>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E15" s="2" t="n">
         <v>0.0</v>
@@ -756,18 +829,21 @@
         <v>0.0</v>
       </c>
       <c r="G15" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H15" s="2" t="n">
         <v>118.0</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I15" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -789,8 +865,10 @@
           <t>1508701192</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
-        <v>0.0</v>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E16" s="2" t="n">
         <v>0.0</v>
@@ -799,18 +877,21 @@
         <v>0.0</v>
       </c>
       <c r="G16" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>49.0</v>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I16" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -832,8 +913,10 @@
           <t>1058807174</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
-        <v>0.0</v>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E17" s="2" t="n">
         <v>0.0</v>
@@ -842,18 +925,21 @@
         <v>0.0</v>
       </c>
       <c r="G17" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>19.0</v>
       </c>
-      <c r="H17" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I17" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -875,8 +961,10 @@
           <t>6258803309</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
-        <v>0.0</v>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E18" s="2" t="n">
         <v>0.0</v>
@@ -885,18 +973,21 @@
         <v>0.0</v>
       </c>
       <c r="G18" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>58.0</v>
       </c>
-      <c r="H18" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I18" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -918,8 +1009,10 @@
           <t>6798502456</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
-        <v>0.0</v>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E19" s="2" t="n">
         <v>0.0</v>
@@ -928,18 +1021,21 @@
         <v>0.0</v>
       </c>
       <c r="G19" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>9.0</v>
       </c>
-      <c r="H19" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I19" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -961,8 +1057,10 @@
           <t>8738702917</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n">
-        <v>0.0</v>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E20" s="2" t="n">
         <v>0.0</v>
@@ -971,18 +1069,21 @@
         <v>0.0</v>
       </c>
       <c r="G20" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>12.0</v>
       </c>
-      <c r="H20" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I20" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1004,8 +1105,10 @@
           <t>1312660786</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n">
-        <v>0.0</v>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E21" s="2" t="n">
         <v>0.0</v>
@@ -1014,18 +1117,21 @@
         <v>0.0</v>
       </c>
       <c r="G21" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>70.0</v>
       </c>
-      <c r="H21" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I21" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1047,28 +1153,33 @@
           <t>1348500111</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n">
-        <v>2.0</v>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E22" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="G22" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>82.0</v>
       </c>
-      <c r="H22" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I22" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1090,8 +1201,10 @@
           <t>1398115533</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n">
-        <v>0.0</v>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E23" s="2" t="n">
         <v>0.0</v>
@@ -1100,18 +1213,21 @@
         <v>0.0</v>
       </c>
       <c r="G23" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>37.0</v>
       </c>
-      <c r="H23" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I23" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1133,8 +1249,10 @@
           <t>1398100699</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
-        <v>0.0</v>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E24" s="2" t="n">
         <v>0.0</v>
@@ -1143,18 +1261,21 @@
         <v>0.0</v>
       </c>
       <c r="G24" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>79.0</v>
       </c>
-      <c r="H24" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I24" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1176,20 +1297,22 @@
           <t>1318629038</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n">
-        <v>80.0</v>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E25" s="2" t="n">
         <v>80.0</v>
       </c>
       <c r="F25" s="2" t="n">
+        <v>80.0</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>47.0</v>
       </c>
-      <c r="G25" s="2" t="n">
-        <v>44.0</v>
-      </c>
       <c r="H25" s="2" t="n">
-        <v>0.0</v>
+        <v>40.0</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>0.0</v>
@@ -1197,7 +1320,10 @@
       <c r="J25" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1219,28 +1345,33 @@
           <t>1348150350</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
-        <v>288.0</v>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E26" s="2" t="n">
         <v>288.0</v>
       </c>
       <c r="F26" s="2" t="n">
+        <v>288.0</v>
+      </c>
+      <c r="G26" s="2" t="n">
         <v>1.0</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>217.0</v>
       </c>
-      <c r="H26" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I26" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J26" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K26" s="2" t="n">
         <v>73.0</v>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1262,28 +1393,33 @@
           <t>1308628716</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n">
-        <v>47.0</v>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E27" s="2" t="n">
         <v>47.0</v>
       </c>
       <c r="F27" s="2" t="n">
+        <v>47.0</v>
+      </c>
+      <c r="G27" s="2" t="n">
         <v>10.0</v>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>27.0</v>
       </c>
-      <c r="H27" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I27" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1305,28 +1441,33 @@
           <t>1378514007</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n">
-        <v>209.0</v>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E28" s="2" t="n">
         <v>209.0</v>
       </c>
       <c r="F28" s="2" t="n">
+        <v>209.0</v>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>92.0</v>
       </c>
-      <c r="G28" s="2" t="n">
-        <v>122.0</v>
-      </c>
       <c r="H28" s="2" t="n">
-        <v>11.0</v>
+        <v>115.0</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>13.0</v>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
+        <v>5.0</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1348,28 +1489,33 @@
           <t>6108128707</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n">
-        <v>157.0</v>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E29" s="2" t="n">
         <v>157.0</v>
       </c>
       <c r="F29" s="2" t="n">
+        <v>157.0</v>
+      </c>
+      <c r="G29" s="2" t="n">
         <v>1.0</v>
       </c>
-      <c r="G29" s="2" t="n">
-        <v>94.0</v>
-      </c>
       <c r="H29" s="2" t="n">
-        <v>2.0</v>
+        <v>65.0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="J29" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K29" s="2" t="n">
         <v>71.0</v>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1391,28 +1537,33 @@
           <t>3128157991</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n">
-        <v>70.0</v>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E30" s="2" t="n">
         <v>70.0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>70.0</v>
+        <v>0.0</v>
       </c>
       <c r="H30" s="2" t="n">
+        <v>80.0</v>
+      </c>
+      <c r="I30" s="2" t="n">
         <v>17.0</v>
       </c>
-      <c r="I30" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="J30" s="2" t="n">
-        <v>49.0</v>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
+        <v>0.0</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>47.0</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1434,8 +1585,10 @@
           <t>1278107419</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n">
-        <v>0.0</v>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>김경훈</t>
+        </is>
       </c>
       <c r="E31" s="2" t="n">
         <v>0.0</v>
@@ -1444,18 +1597,21 @@
         <v>0.0</v>
       </c>
       <c r="G31" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H31" s="2" t="n">
         <v>103.0</v>
       </c>
-      <c r="H31" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1477,28 +1633,33 @@
           <t>5158140973</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
-        <v>194.0</v>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>한규범 외 5명</t>
+        </is>
       </c>
       <c r="E32" s="2" t="n">
         <v>194.0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.0</v>
+        <v>194.0</v>
       </c>
       <c r="G32" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H32" s="2" t="n">
         <v>169.0</v>
       </c>
-      <c r="H32" s="2" t="n">
-        <v>11.0</v>
-      </c>
       <c r="I32" s="2" t="n">
-        <v>16.0</v>
+        <v>12.0</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
+        <v>14.0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1520,8 +1681,10 @@
           <t>1138156416</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n">
-        <v>0.0</v>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E33" s="2" t="n">
         <v>0.0</v>
@@ -1530,18 +1693,21 @@
         <v>0.0</v>
       </c>
       <c r="G33" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H33" s="2" t="n">
         <v>35.0</v>
       </c>
-      <c r="H33" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I33" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1563,8 +1729,10 @@
           <t>1348106311</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n">
-        <v>0.0</v>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E34" s="2" t="n">
         <v>0.0</v>
@@ -1573,18 +1741,21 @@
         <v>0.0</v>
       </c>
       <c r="G34" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H34" s="2" t="n">
         <v>286.0</v>
       </c>
-      <c r="H34" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I34" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1606,28 +1777,33 @@
           <t>1208731282</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n">
-        <v>5.0</v>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E35" s="2" t="n">
         <v>5.0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>70.0</v>
+        <v>0.0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0.0</v>
+        <v>67.0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1649,28 +1825,33 @@
           <t>6131783159</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
-        <v>452.0</v>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>송민규 외 5명</t>
+        </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>315.0</v>
+        <v>476.0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.0</v>
+        <v>339.0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>234.0</v>
+        <v>0.0</v>
       </c>
       <c r="H36" s="2" t="n">
+        <v>205.0</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="J36" s="2" t="n">
         <v>22.0</v>
       </c>
-      <c r="I36" s="2" t="n">
-        <v>41.0</v>
-      </c>
-      <c r="J36" s="2" t="n">
-        <v>17.0</v>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1692,8 +1873,10 @@
           <t>1228159023</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n">
-        <v>0.0</v>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>이승건</t>
+        </is>
       </c>
       <c r="E37" s="2" t="n">
         <v>0.0</v>
@@ -1702,18 +1885,21 @@
         <v>0.0</v>
       </c>
       <c r="G37" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H37" s="2" t="n">
         <v>41.0</v>
       </c>
-      <c r="H37" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I37" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1735,28 +1921,33 @@
           <t>7758501361</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n">
-        <v>163.0</v>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>이승건</t>
+        </is>
       </c>
       <c r="E38" s="2" t="n">
         <v>163.0</v>
       </c>
       <c r="F38" s="2" t="n">
+        <v>163.0</v>
+      </c>
+      <c r="G38" s="2" t="n">
         <v>16.0</v>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="H38" s="2" t="n">
         <v>10.0</v>
       </c>
-      <c r="H38" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I38" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1778,28 +1969,33 @@
           <t>1018156320</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n">
-        <v>45.0</v>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>정경훈</t>
+        </is>
       </c>
       <c r="E39" s="2" t="n">
         <v>45.0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.0</v>
+        <v>45.0</v>
       </c>
       <c r="G39" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H39" s="2" t="n">
         <v>150.0</v>
       </c>
-      <c r="H39" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I39" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1821,28 +2017,33 @@
           <t>1378604165</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n">
-        <v>237.0</v>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E40" s="2" t="n">
         <v>237.0</v>
       </c>
       <c r="F40" s="2" t="n">
+        <v>237.0</v>
+      </c>
+      <c r="G40" s="2" t="n">
         <v>57.0</v>
       </c>
-      <c r="G40" s="2" t="n">
-        <v>183.0</v>
-      </c>
       <c r="H40" s="2" t="n">
-        <v>30.0</v>
+        <v>156.0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>27.0</v>
+        <v>15.0</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>86.0</v>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
+        <v>24.0</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>113.0</v>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1864,28 +2065,33 @@
           <t>1198678150</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n">
-        <v>10.0</v>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>정경훈</t>
+        </is>
       </c>
       <c r="E41" s="2" t="n">
         <v>10.0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G41" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H41" s="2" t="n">
         <v>160.0</v>
       </c>
-      <c r="H41" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I41" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1907,28 +2113,33 @@
           <t>3148613655</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n">
-        <v>60.0</v>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>송민규 외 5명</t>
+        </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>60.0</v>
+        <v>61.0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>16.0</v>
+        <v>61.0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>23.0</v>
+        <v>17.0</v>
       </c>
       <c r="H42" s="2" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="I42" s="2" t="n">
         <v>4.0</v>
       </c>
-      <c r="I42" s="2" t="n">
+      <c r="J42" s="2" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="K42" s="2" t="n">
         <v>1.0</v>
       </c>
-      <c r="J42" s="2" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1950,28 +2161,33 @@
           <t>3128109219</t>
         </is>
       </c>
-      <c r="D43" s="2" t="n">
-        <v>1827.0</v>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E43" s="2" t="n">
         <v>1827.0</v>
       </c>
       <c r="F43" s="2" t="n">
+        <v>1827.0</v>
+      </c>
+      <c r="G43" s="2" t="n">
         <v>525.0</v>
       </c>
-      <c r="G43" s="2" t="n">
-        <v>936.0</v>
-      </c>
       <c r="H43" s="2" t="n">
-        <v>3.0</v>
+        <v>920.0</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="J43" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K43" s="2" t="n">
         <v>18.0</v>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1993,28 +2209,33 @@
           <t>1128138619</t>
         </is>
       </c>
-      <c r="D44" s="2" t="n">
-        <v>84.0</v>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E44" s="2" t="n">
         <v>84.0</v>
       </c>
       <c r="F44" s="2" t="n">
+        <v>84.0</v>
+      </c>
+      <c r="G44" s="2" t="n">
         <v>22.0</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="H44" s="2" t="n">
         <v>70.0</v>
       </c>
-      <c r="H44" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I44" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2036,28 +2257,33 @@
           <t>6088151660</t>
         </is>
       </c>
-      <c r="D45" s="2" t="n">
-        <v>1184.0</v>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>허세헌 외 5명</t>
+        </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1165.0</v>
+        <v>1202.0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>28.0</v>
+        <v>1183.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1521.0</v>
+        <v>29.0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>0.0</v>
+        <v>1519.0</v>
       </c>
       <c r="I45" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J45" s="2" t="n">
         <v>39.0</v>
       </c>
-      <c r="J45" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2079,28 +2305,33 @@
           <t>1258112293</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n">
-        <v>614.0</v>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E46" s="2" t="n">
         <v>614.0</v>
       </c>
       <c r="F46" s="2" t="n">
+        <v>614.0</v>
+      </c>
+      <c r="G46" s="2" t="n">
         <v>250.0</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="H46" s="2" t="n">
         <v>319.0</v>
       </c>
-      <c r="H46" s="2" t="n">
-        <v>2.0</v>
-      </c>
       <c r="I46" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J46" s="2" t="n">
         <v>9.0</v>
       </c>
-      <c r="J46" s="2" t="n">
-        <v>376.0</v>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="n">
+        <v>377.0</v>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2122,28 +2353,33 @@
           <t>1238106174</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n">
-        <v>916.0</v>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
       </c>
       <c r="E47" s="2" t="n">
         <v>916.0</v>
       </c>
       <c r="F47" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="G47" s="2" t="n">
         <v>128.0</v>
       </c>
-      <c r="G47" s="2" t="n">
-        <v>839.0</v>
-      </c>
       <c r="H47" s="2" t="n">
-        <v>117.0</v>
+        <v>837.0</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>21.0</v>
+        <v>109.0</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>163.0</v>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
+        <v>43.0</v>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>179.0</v>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2165,28 +2401,33 @@
           <t>3128564374</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n">
-        <v>85.0</v>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
       </c>
       <c r="E48" s="2" t="n">
         <v>85.0</v>
       </c>
       <c r="F48" s="2" t="n">
+        <v>85.0</v>
+      </c>
+      <c r="G48" s="2" t="n">
         <v>5.0</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="H48" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="H48" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I48" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
data: update 고객사계측기현황.xlsx for 2026-09-23
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사계측기현황.xlsx
+++ b/docs/dashboard/data/고객사계측기현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -180,44 +180,44 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>한국의료기기평가원</t>
+          <t>로타렉스코리아 주식회사</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>경기도 성남시 분당구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1298210386</t>
+          <t>6898101887</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>한윤규 외 1명</t>
+          <t>이선재 외 1명</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0</v>
+        <v>748.0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0</v>
+        <v>748.0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.0</v>
+        <v>574.0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>136.0</v>
+        <v>474.0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.0</v>
+        <v>9.0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0.0</v>
+        <v>32.0</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -228,44 +228,44 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>굴드펌프(주)</t>
+          <t>(주)광일테크</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>충청북도 청주시 흥덕구</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2118642792</t>
+          <t>3108118935</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>이선재 외 1명</t>
+          <t>신승호</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>192.0</v>
+        <v>2.0</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -276,44 +276,44 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>하이에어코리아(주)</t>
+          <t>(주) 신우테크</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>경상남도 김해시</t>
+          <t xml:space="preserve">세종특별자치시 </t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>6038110081</t>
+          <t>1258137969</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>한규범 외 5명</t>
+          <t>신승호</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>467.0</v>
+        <v>0.0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>467.0</v>
+        <v>0.0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>15.0</v>
+        <v>0.0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>421.0</v>
+        <v>1.0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>24.0</v>
+        <v>0.0</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>15.0</v>
+        <v>0.0</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>136.0</v>
+        <v>0.0</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -324,35 +324,35 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>한국의료기기평가원</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>경기도 성남시 수정구</t>
+          <t>경기도 성남시 분당구</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>1298210386</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>한윤규</t>
+          <t>한윤규 외 1명</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>119.0</v>
+        <v>0.0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>99.0</v>
+        <v>0.0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>99.0</v>
+        <v>0.0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>178.0</v>
+        <v>136.0</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0.0</v>
@@ -361,7 +361,7 @@
         <v>0.0</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
@@ -372,44 +372,44 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>현대건설(주)</t>
+          <t>굴드펌프(주)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>경상북도 울진군</t>
+          <t>충청북도 청주시 흥덕구</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1018116293</t>
+          <t>2118642792</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이선재 외 1명</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>4.0</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="H6" s="2" t="n">
+        <v>209.0</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="K6" s="2" t="n">
         <v>4.0</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>30.0</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>0.0</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -420,44 +420,44 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경상남도 김해시</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>송민규 외 5명</t>
+          <t>한규범 외 5명</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0</v>
+        <v>467.0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.0</v>
+        <v>467.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.0</v>
+        <v>15.0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>19.0</v>
+        <v>473.0</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0.0</v>
+        <v>136.0</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -468,35 +468,35 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>한윤규</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0</v>
+        <v>119.0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.0</v>
+        <v>99.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.0</v>
+        <v>99.0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>37.0</v>
+        <v>178.0</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0.0</v>
@@ -505,7 +505,7 @@
         <v>0.0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
@@ -516,35 +516,35 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>전원준 외 1명</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>10.0</v>
+        <v>4.0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>10.0</v>
+        <v>4.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>166.0</v>
+        <v>30.0</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0.0</v>
@@ -564,35 +564,35 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>송민규 외 5명</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>44.0</v>
+        <v>0.0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>44.0</v>
+        <v>0.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>43.0</v>
+        <v>0.0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>40.0</v>
+        <v>19.0</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0.0</v>
@@ -601,7 +601,7 @@
         <v>0.0</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -612,17 +612,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -631,25 +631,25 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>293.0</v>
+        <v>0.0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>293.0</v>
+        <v>0.0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>54.0</v>
+        <v>0.0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>231.0</v>
+        <v>37.0</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>30.0</v>
+        <v>0.0</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>19.0</v>
+        <v>0.0</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>227.0</v>
+        <v>0.0</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -660,35 +660,35 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>전원준 외 1명</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>223.0</v>
+        <v>163.0</v>
       </c>
       <c r="I12" s="2" t="n">
         <v>0.0</v>
@@ -708,17 +708,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -727,16 +727,16 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0</v>
+        <v>44.0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.0</v>
+        <v>44.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.0</v>
+        <v>43.0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23.0</v>
+        <v>40.0</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>0.0</v>
@@ -745,7 +745,7 @@
         <v>0.0</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
@@ -756,17 +756,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -775,25 +775,25 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.0</v>
+        <v>54.0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>30.0</v>
+        <v>231.0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.0</v>
+        <v>21.0</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0.0</v>
+        <v>227.0</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
@@ -804,22 +804,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -832,7 +832,7 @@
         <v>0.0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>118.0</v>
+        <v>223.0</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>0.0</v>
@@ -852,22 +852,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -880,7 +880,7 @@
         <v>0.0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>49.0</v>
+        <v>23.0</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>0.0</v>
@@ -900,22 +900,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -928,7 +928,7 @@
         <v>0.0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>19.0</v>
+        <v>30.0</v>
       </c>
       <c r="I17" s="2" t="n">
         <v>0.0</v>
@@ -948,17 +948,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
         <v>0.0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>58.0</v>
+        <v>118.0</v>
       </c>
       <c r="I18" s="2" t="n">
         <v>0.0</v>
@@ -996,17 +996,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1024,7 +1024,7 @@
         <v>0.0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>9.0</v>
+        <v>49.0</v>
       </c>
       <c r="I19" s="2" t="n">
         <v>0.0</v>
@@ -1044,17 +1044,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
         <v>0.0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>12.0</v>
+        <v>19.0</v>
       </c>
       <c r="I20" s="2" t="n">
         <v>0.0</v>
@@ -1092,17 +1092,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1120,7 +1120,7 @@
         <v>0.0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>70.0</v>
+        <v>58.0</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>0.0</v>
@@ -1140,17 +1140,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1159,16 +1159,16 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>82.0</v>
+        <v>9.0</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0.0</v>
@@ -1188,17 +1188,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
         <v>0.0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>37.0</v>
+        <v>12.0</v>
       </c>
       <c r="I23" s="2" t="n">
         <v>0.0</v>
@@ -1236,7 +1236,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1264,7 +1264,7 @@
         <v>0.0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>79.0</v>
+        <v>58.0</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>0.0</v>
@@ -1284,17 +1284,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1303,16 +1303,16 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>80.0</v>
+        <v>2.0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>80.0</v>
+        <v>2.0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>47.0</v>
+        <v>0.0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>40.0</v>
+        <v>82.0</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>0.0</v>
@@ -1332,35 +1332,35 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>288.0</v>
+        <v>0.0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>288.0</v>
+        <v>0.0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>217.0</v>
+        <v>37.0</v>
       </c>
       <c r="I26" s="2" t="n">
         <v>0.0</v>
@@ -1369,7 +1369,7 @@
         <v>0.0</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>73.0</v>
+        <v>0.0</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -1380,7 +1380,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1399,16 +1399,16 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>47.0</v>
+        <v>0.0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>47.0</v>
+        <v>0.0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>27.0</v>
+        <v>79.0</v>
       </c>
       <c r="I27" s="2" t="n">
         <v>0.0</v>
@@ -1428,17 +1428,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1447,25 +1447,25 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>209.0</v>
+        <v>80.0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>209.0</v>
+        <v>80.0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>92.0</v>
+        <v>47.0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>115.0</v>
+        <v>40.0</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>18.0</v>
+        <v>0.0</v>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -1476,17 +1476,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1495,25 +1495,25 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>157.0</v>
+        <v>288.0</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>157.0</v>
+        <v>288.0</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>65.0</v>
+        <v>284.0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>71.0</v>
+        <v>73.0</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -1524,44 +1524,44 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>70.0</v>
+        <v>47.0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>70.0</v>
+        <v>47.0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>80.0</v>
+        <v>44.0</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>47.0</v>
+        <v>0.0</v>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
@@ -1572,44 +1572,44 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>김경훈</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0</v>
+        <v>209.0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.0</v>
+        <v>209.0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.0</v>
+        <v>92.0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>103.0</v>
+        <v>114.0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.0</v>
+        <v>9.0</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -1620,44 +1620,44 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>한규범 외 5명</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>194.0</v>
+        <v>157.0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>194.0</v>
+        <v>157.0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>169.0</v>
+        <v>40.0</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>12.0</v>
+        <v>1.0</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>14.0</v>
+        <v>1.0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>6.0</v>
+        <v>71.0</v>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
@@ -1668,44 +1668,44 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>35.0</v>
+        <v>80.0</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.0</v>
+        <v>15.0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0.0</v>
+        <v>47.0</v>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
@@ -1716,22 +1716,22 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>김경훈</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -1744,7 +1744,7 @@
         <v>0.0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>286.0</v>
+        <v>103.0</v>
       </c>
       <c r="I34" s="2" t="n">
         <v>0.0</v>
@@ -1764,44 +1764,44 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>한규범 외 5명</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>5.0</v>
+        <v>194.0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>5.0</v>
+        <v>194.0</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>67.0</v>
+        <v>160.0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.0</v>
+        <v>15.0</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
@@ -1812,44 +1812,44 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>송민규 외 5명</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>476.0</v>
+        <v>0.0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>339.0</v>
+        <v>0.0</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>205.0</v>
+        <v>35.0</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>22.0</v>
+        <v>0.0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>40.0</v>
+        <v>0.0</v>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
@@ -1860,22 +1860,22 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>이승건</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -1888,7 +1888,7 @@
         <v>0.0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>41.0</v>
+        <v>286.0</v>
       </c>
       <c r="I37" s="2" t="n">
         <v>0.0</v>
@@ -1908,35 +1908,35 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>이승건</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>163.0</v>
+        <v>5.0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>163.0</v>
+        <v>5.0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>10.0</v>
+        <v>67.0</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>0.0</v>
@@ -1956,44 +1956,44 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>송민규 외 5명</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>45.0</v>
+        <v>476.0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>45.0</v>
+        <v>339.0</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>150.0</v>
+        <v>205.0</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0.0</v>
+        <v>39.0</v>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
@@ -2004,44 +2004,44 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>이승건</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>237.0</v>
+        <v>0.0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>237.0</v>
+        <v>0.0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>57.0</v>
+        <v>0.0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>156.0</v>
+        <v>41.0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>15.0</v>
+        <v>0.0</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>24.0</v>
+        <v>0.0</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>113.0</v>
+        <v>0.0</v>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
@@ -2052,35 +2052,35 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>이승건</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
+        <v>163.0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>163.0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="H41" s="2" t="n">
         <v>10.0</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="G41" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H41" s="2" t="n">
-        <v>160.0</v>
       </c>
       <c r="I41" s="2" t="n">
         <v>0.0</v>
@@ -2100,44 +2100,44 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>송민규 외 5명</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>61.0</v>
+        <v>45.0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>61.0</v>
+        <v>45.0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>22.0</v>
+        <v>150.0</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
@@ -2148,44 +2148,44 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1827.0</v>
+        <v>237.0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>1827.0</v>
+        <v>237.0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>525.0</v>
+        <v>57.0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>920.0</v>
+        <v>156.0</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>4.0</v>
+        <v>17.0</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>18.0</v>
+        <v>113.0</v>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -2196,35 +2196,35 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>84.0</v>
+        <v>10.0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>84.0</v>
+        <v>10.0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>22.0</v>
+        <v>0.0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>70.0</v>
+        <v>159.0</v>
       </c>
       <c r="I44" s="2" t="n">
         <v>0.0</v>
@@ -2244,41 +2244,41 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>허세헌 외 5명</t>
+          <t>송민규 외 5명</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1202.0</v>
+        <v>61.0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1183.0</v>
+        <v>61.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>29.0</v>
+        <v>17.0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1519.0</v>
+        <v>22.0</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>39.0</v>
+        <v>4.0</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0.0</v>
@@ -2292,17 +2292,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2311,25 +2311,25 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>614.0</v>
+        <v>1827.0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>614.0</v>
+        <v>1827.0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>250.0</v>
+        <v>525.0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>319.0</v>
+        <v>919.0</v>
       </c>
       <c r="I46" s="2" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="J46" s="2" t="n">
         <v>1.0</v>
       </c>
-      <c r="J46" s="2" t="n">
-        <v>9.0</v>
-      </c>
       <c r="K46" s="2" t="n">
-        <v>377.0</v>
+        <v>18.0</v>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
@@ -2340,17 +2340,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2359,25 +2359,25 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>916.0</v>
+        <v>84.0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>916.0</v>
+        <v>84.0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>128.0</v>
+        <v>22.0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>837.0</v>
+        <v>69.0</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>109.0</v>
+        <v>0.0</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>43.0</v>
+        <v>0.0</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>179.0</v>
+        <v>0.0</v>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
@@ -2388,46 +2388,190 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>(주)신화프리텍</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>경남 창원시 성산구</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>6088151660</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>허세헌 외 5명</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1207.0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>1188.0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>29.0</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>1518.0</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>39.0</v>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>(주)한국기능공사</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>충북 음성군</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>1258112293</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>614.0</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>614.0</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>250.0</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>310.0</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>383.0</v>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>(주)휴니드테크놀러지스</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>인천 연수구</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>1238106174</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>정상훈</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>128.0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>837.0</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>110.0</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>43.0</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>179.0</v>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
           <t>(주)서연이화 아산공장</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>충남 아산시</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>3128564374</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>전원준</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="E51" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F51" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>5.0</v>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="H51" s="2" t="n">
         <v>85.0</v>
       </c>
-      <c r="I48" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J48" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K48" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="I51" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>